<commit_message>
Parte 6c: operador fuera del sitio público (sin sigla en detalle/cards/schema/llms), esteros-del-ibera inactivo hasta tener base doble, base single en Salta & Purmamarca y Valle de la Luna, 4 fotos sin repetir por región
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -2364,7 +2364,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>INACTIVO: falta precio por persona base doble</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 1.395.002 (por persona en base doble — total con impuestos)
+          <t>Desde ARS 1.395.002 (por persona en base single — total con impuestos)
 Precio total por persona publicado por el operador para 1 adulto (incluye impuestos), fecha de ejemplo 17–20 nov 2026. Salidas diarias: la ficha no da fecha límite, se carga vigencia 31/12/2026 para revisión.
 single: ARS 1.395.002</t>
         </is>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 1.362.212 (por persona en base doble — total con impuestos)
+          <t>Desde ARS 1.362.212 (por persona en base single — total con impuestos)
 Precio total por persona publicado por el operador para 1 adulto (incluye impuestos); no publica base doble.
 single: ARS 1.362.212</t>
         </is>

</xml_diff>

<commit_message>
Parte 6d — All Seasons (AS-322357, AS-561135, AS-561130, AS-195199, AS-217217, AS-118771, AS-162781): 7 paquetes nuevos de Brasil; filas en la planilla de revisión
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisión parte 6" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Revisión parte 6'!$A$1:$O$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Revisión parte 6'!$A$1:$O$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3371,8 +3371,487 @@
       <c r="N41" s="2" t="inlineStr"/>
       <c r="O41" s="2" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Búzios — 9 de enero 2027</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>https://allseasons.tourvector.com/espanol/paquete2/561135/Descubri-Buzios-con-JetSMART/194626755/</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>9 de enero 2027</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Búzios: Lestada Pousada · 7 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>JetSMART JA 3816 Buenos Aires (EZE) – Río de Janeiro 09/01/2027 12:54 – 15:50
+JetSMART JA 3817 Río de Janeiro – Buenos Aires (EZE) 16/01/2027 13:50 – 17:14</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>1 valija de 23 kg en bodega</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 1.500 (por persona en base doble — precio final con impuestos)
+Precio final por persona en base doble publicado por el operador: USD 1.500 (total 2 adultos USD 3.000). La ficha no desglosa componentes.</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-09</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hotel; confirmar que es precio de venta al público</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Río de Janeiro — 9 de enero 2027</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>https://allseasons.tourvector.com/espanol/paquete2/561130/Disfruta-Rio-De-Janeiro-con-JetSMART/193847595/</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>9 de enero 2027</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Río de Janeiro (Copacabana): Windsor Martinique 3* · 7 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>JetSMART JA 3816 Buenos Aires (EZE) – Río de Janeiro 09/01/2027 12:54 – 15:50
+JetSMART JA 3817 Río de Janeiro – Buenos Aires (EZE) 16/01/2027 13:50 – 17:14</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>1 valija de 23 kg en bodega</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 1.500 (por persona en base doble — precio final con impuestos)
+Precio final por persona en base doble publicado por el operador: USD 1.500 (total 2 adultos USD 3.000). La ficha no desglosa componentes.</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-09</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>confirmar que es precio de venta al público</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Salvador de Bahía — 9 de enero 2027</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>https://allseasons.tourvector.com/espanol/paquete2/217217/Salvador-con-GOL/193685985/</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>9 de enero 2027</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Salvador de Bahía (Ondina): Vila Galé Salvador 5* · 7 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>GOL G3 7213 Buenos Aires (AEP) – Salvador (SSA) 09/01/2027 22:15 – 02:40 (+1)
+GOL G3 7212 Salvador (SSA) – Buenos Aires (AEP) 17/01/2027 03:10 – 08:00</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>1 valija de 23 kg en bodega</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 1.356 (por persona en base doble — precio final con impuestos)
+Precio final por persona en base doble publicado por el operador: USD 1.356 (total 2 adultos USD 2.712). La ficha no desglosa componentes. Otras salidas listadas sin precio: enero a marzo 2027.</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-09</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>otras fechas sin precio; confirmar que es precio de venta al público</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Arraial d'Ajuda — 10 de enero 2027</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>https://allseasons.tourvector.com/espanol/paquete2/322357/Arraial-DAjuda-con-GOL/194999179/</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>10 de enero 2027</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Arraial d'Ajuda: Pousada Coqueiros · 7 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>GOL G3 7493 Buenos Aires (EZE) – Porto Seguro (BPS) 10/01/2027 01:10 – 05:00
+GOL G3 7492 Porto Seguro (BPS) – Buenos Aires (EZE) 16/01/2027 23:00 – 03:10 (+1)</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>1 valija de 23 kg en bodega</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 1.739 (por persona en base doble — precio final con impuestos)
+Precio final por persona en base doble publicado por el operador: USD 1.739 (total 2 adultos USD 3.478). La ficha no desglosa componentes. Otras salidas listadas sin precio: 17/01/2027.</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-10</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hotel; otras fechas sin precio; confirmar que es precio de venta al público</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Florianópolis — 16 de enero 2027</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>https://allseasons.tourvector.com/espanol/paquete2/118771/Descubri-Florianopolis-con-JetSMART/194950084/</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>16 de enero 2027</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Florianópolis (Ingleses): Porto Sol Ingleses · 7 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>JetSMART JA 3824 Buenos Aires (EZE) – Florianópolis (FLN) 16/01/2027 12:15 – 14:15
+JetSMART JA 3825 Florianópolis (FLN) – Buenos Aires (EZE) 23/01/2027 15:10 – 17:25</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>1 valija de 23 kg en bodega</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 1.480 (por persona en base doble — precio final con impuestos)
+Precio final por persona en base doble publicado por el operador: USD 1.480 (total 2 adultos USD 2.960). La ficha no desglosa componentes. Otras salidas listadas sin precio: 09/01/2027.</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-16</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hotel; otras fechas sin precio; confirmar que es precio de venta al público</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Maceió — 26 de enero 2027</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>https://allseasons.tourvector.com/espanol/paquete2/195199/Descubri-Maceio-con-LATAM/195126896/</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>26 de enero 2027</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Maceió: Ritz Suites Grand Hotel Boutique · 7 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>LATAM LA 8163 Buenos Aires (EZE) – Maceió (MCZ) 26/01/2027 02:15 – 07:15
+LATAM LA 8162 Maceió (MCZ) – Buenos Aires (EZE) 02/02/2027 10:45 – 16:00</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>1 valija de 23 kg en bodega</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 1.511 (por persona en base doble — precio final con impuestos)
+Precio final por persona en base doble publicado por el operador: USD 1.511 (total 2 adultos USD 3.022). La ficha no desglosa componentes. Otras salidas listadas sin precio: 12/01/2027 y 19/01/2027.</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-26</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hotel; otras fechas sin precio; confirmar que es precio de venta al público</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Praia do Forte — 20 de febrero 2027</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>20 de febrero 2027</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Praia do Forte: Iberostar Waves Bahia · 7 noches · All Inclusive</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>GOL G3 7213 Buenos Aires (AEP) – Salvador (SSA) 20/02/2027 22:00 – 02:10 (+1)
+GOL G3 7212 Salvador (SSA) – Buenos Aires (AEP) 28/02/2027 03:10 – 08:00</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>1 valija de 23 kg en bodega</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 2.537 (por persona en base doble — precio final con impuestos)
+Precio final por persona en base doble publicado por el operador: USD 2.537 (total 2 adultos USD 5.074). La ficha no desglosa componentes. Otras salidas listadas sin precio: enero a marzo 2027.</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>2027-02-20</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hotel; otras fechas sin precio; confirmar que es precio de venta al público</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O41"/>
+  <autoFilter ref="A1:O48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Parte 6e (decisiones del usuario): Cuarto Continente con precio estimado 'Desde' y fecha a elección hasta julio 2027; Mágicamente Europa (JT-2193) con el precio de la ficha y tasas hoteleras aparte; Sudáfrica & Mauritius queda con la salida del 8/2/2027; se elimina esteros-del-ibera
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -660,7 +660,7 @@
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Desde USD 9.820 (por persona en base doble — total con impuestos)
-Base doble USD 7.950 + impuestos USD 1.870 (DNT, IVA, gastos y propinas) = USD 9.820. Single: 7.950 + 2.880 + 1.870 = 12.700. Los vuelos de la ficha figuran con fechas de noviembre (16NOV–28NOV): se cargan solo aerolínea, ruta y número.
+Base doble USD 7.950 + impuestos USD 1.870 (DNT, IVA, gastos y propinas) = USD 9.820. Single: 7.950 + 2.880 + 1.870 = 12.700. Los vuelos de la ficha figuran con fechas de noviembre (16NOV–28NOV): se cargan solo aerolínea, ruta y número. Decisión del usuario (15/10/2026): se publica la salida del 8 de febrero 2027.
 single: USD 12.700</t>
         </is>
       </c>
@@ -1992,8 +1992,8 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Desde USD 4.622 (por persona en base doble — tarifa + impuestos + IVA/gastos + tasas hoteleras)
-Tarifa USD 3.696 + impuestos aéreos USD 582 + IVA y gastos USD 248 = USD 4.526, más tasas hoteleras obligatorias USD 94 + USD 2 de gastos (se pagan al reservar) = USD 4.622. Triple y single: consultar. Seña USD 2.100.</t>
+          <t>Desde USD 4.526 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
+Tarifa USD 3.696 + impuestos aéreos USD 582 + IVA y gastos USD 248 = USD 4.526 (como publica la ficha). Tasas hoteleras obligatorias USD 94 + USD 2 de gastos aparte, se pagan al reservar. Triple y single: consultar. Seña USD 2.100.</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Escapada a Mendoza — 27 de octubre 2026</t>
+          <t>Escapada a Mendoza</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>27 de octubre 2026</t>
+          <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
@@ -2050,8 +2050,8 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Aerolíneas Argentinas AR 1402 Buenos Aires (AEP) – Mendoza 27/10/2026 07:40 – 09:40
-Aerolíneas Argentinas AR 1401 Mendoza – Buenos Aires (AEP) 30/10/2026 07:30 – 09:10</t>
+          <t>Aerolíneas Argentinas AR 1402 Buenos Aires (AEP) – Mendoza 07:40 – 09:40
+Aerolíneas Argentinas AR 1401 Mendoza – Buenos Aires (AEP) 07:30 – 09:10</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -2061,8 +2061,8 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 567.676 (por persona en base doble — total con impuestos)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes.</t>
+          <t>Desde ARS 567.676 (por persona en base doble — precio estimado, se cotiza al consultar)
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2072,12 +2072,12 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2027-07-31</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>categoría de algunos hoteles; itinerario día por día (la ficha no lo tiene)</t>
+          <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
@@ -2096,17 +2096,17 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Bariloche lo tiene todo — 27 de octubre 2026</t>
+          <t>Ushuaia</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://cuartocontinente.com/es/idea/40420928/bariloche-lo-tiene-todo?country=AR</t>
+          <t>https://cuartocontinente.com/es/idea/22203065/ushuaia?country=AR</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>27 de octubre 2026</t>
+          <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -2114,13 +2114,13 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Bariloche: Hotel Nevada · 3 noches · Desayuno</t>
+          <t>Ushuaia: Del Bosque Apart &amp; Hotel · 3 noches · Desayuno</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Aerolíneas Argentinas AR 1680 Buenos Aires (AEP) – Bariloche 27/10/2026 04:35 – 07:00
-Aerolíneas Argentinas AR 1681 Bariloche – Buenos Aires (AEP) 30/10/2026 11:55 – 14:00</t>
+          <t>Aerolíneas Argentinas AR 1886 Buenos Aires (AEP) – Ushuaia 05:50 – 09:30
+Aerolíneas Argentinas AR 1871 Ushuaia – Buenos Aires (AEP) 08:20 – 11:50</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -2130,8 +2130,8 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 651.624 (por persona en base doble — total con impuestos)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes.</t>
+          <t>Desde ARS 949.630 (por persona en base doble — precio estimado, se cotiza al consultar)
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2141,12 +2141,12 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2027-07-31</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>categoría de algunos hoteles; itinerario día por día (la ficha no lo tiene)</t>
+          <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
@@ -2165,17 +2165,17 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Ushuaia — 16 de noviembre 2026</t>
+          <t>Bariloche lo tiene todo</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://cuartocontinente.com/es/idea/22203065/ushuaia?country=AR</t>
+          <t>https://cuartocontinente.com/es/idea/40420928/bariloche-lo-tiene-todo?country=AR</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>16 de noviembre 2026</t>
+          <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -2183,13 +2183,13 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Ushuaia: Del Bosque Apart &amp; Hotel · 3 noches · Desayuno</t>
+          <t>Bariloche: Hotel Nevada · 3 noches · Desayuno</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Aerolíneas Argentinas AR 1886 Buenos Aires (AEP) – Ushuaia 16/11/2026 05:50 – 09:30
-Aerolíneas Argentinas AR 1871 Ushuaia – Buenos Aires (AEP) 19/11/2026 08:20 – 11:50</t>
+          <t>Aerolíneas Argentinas AR 1680 Buenos Aires (AEP) – Bariloche 04:35 – 07:00
+Aerolíneas Argentinas AR 1681 Bariloche – Buenos Aires (AEP) 11:55 – 14:00</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2199,8 +2199,8 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 949.630 (por persona en base doble — total con impuestos)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes.</t>
+          <t>Desde ARS 651.624 (por persona en base doble — precio estimado, se cotiza al consultar)
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2210,12 +2210,12 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2027-07-31</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>categoría de algunos hoteles; itinerario día por día (la ficha no lo tiene)</t>
+          <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Vuelta al norte argentino — 16 de noviembre 2026</t>
+          <t>Vuelta al norte argentino</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>16 de noviembre 2026</t>
+          <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -2259,8 +2259,8 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Aerolíneas Argentinas AR 1468 Buenos Aires (AEP) – Tucumán 16/11/2026 04:55 – 06:55
-Aerolíneas Argentinas AR 1489 Salta – Buenos Aires (AEP) 22/11/2026 08:05 – 10:10</t>
+          <t>Aerolíneas Argentinas AR 1468 Buenos Aires (AEP) – Tucumán 04:55 – 06:55
+Aerolíneas Argentinas AR 1489 Salta – Buenos Aires (AEP) 08:05 – 10:10</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2270,8 +2270,8 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 1.280.826 (por persona en base doble — total con impuestos)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes.</t>
+          <t>Desde ARS 1.280.826 (por persona en base doble — precio estimado, se cotiza al consultar)
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2281,12 +2281,12 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2027-07-31</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>categoría de algunos hoteles</t>
+          <t>categoría de algunos hoteles; fecha/horario de vuelos</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
@@ -2305,31 +2305,33 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Puerto Madryn — 23 de noviembre 2026</t>
+          <t>Ushuaia &amp; El Calafate</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://cuartocontinente.com/es/idea/37028317/puerto-madryn?country=AR</t>
+          <t>https://cuartocontinente.com/es/idea/22204583/ushuaia-el-calafate?country=AR</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>23 de noviembre 2026</t>
+          <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Puerto Madryn: Parry Hotel · 3 noches · Desayuno</t>
+          <t>Ushuaia: Hotel Rosa de los Vientos · 3 noches · Desayuno
+El Calafate: Kapenke Hotel · 3 noches · Desayuno</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Aerolíneas Argentinas AR 1812 Buenos Aires (AEP) – Puerto Madryn 23/11/2026 16:00 – 18:05
-Aerolíneas Argentinas AR 1813 Puerto Madryn – Buenos Aires (AEP) 26/11/2026 19:05 – 20:55</t>
+          <t>Aerolíneas Argentinas AR 1876 Buenos Aires (AEP) – Ushuaia 05:05 – 08:45
+Aerolíneas Argentinas AR 1895 Ushuaia – El Calafate 09:20 – 10:40
+Aerolíneas Argentinas AR 1899 El Calafate – Buenos Aires (AEP) 18:40 – 21:40</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2339,8 +2341,8 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 676.299 (por persona en base doble — total con impuestos)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes.</t>
+          <t>Desde ARS 1.342.389 (por persona en base doble — precio estimado, se cotiza al consultar)
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2350,12 +2352,12 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2027-07-31</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>categoría de algunos hoteles; itinerario día por día (la ficha no lo tiene)</t>
+          <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr"/>
@@ -2364,7 +2366,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>INACTIVO: falta precio por persona base doble</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2374,17 +2376,17 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Esteros del Iberá — 23 de noviembre 2026</t>
+          <t>Puerto Madryn</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://cuartocontinente.com/es/idea/64460563/esteros-del-ibera?country=AR</t>
+          <t>https://cuartocontinente.com/es/idea/37028317/puerto-madryn?country=AR</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>23 de noviembre 2026</t>
+          <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -2392,24 +2394,24 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Colonia Carlos Pellegrini: Posada Ypa Sapukai · 3 noches · Media pensión</t>
+          <t>Puerto Madryn: Parry Hotel · 3 noches · Desayuno</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Aerolíneas Argentinas AR 1764 Buenos Aires (AEP) – Posadas 23/11/2026 13:50 – 15:30
-Aerolíneas Argentinas AR 1769 Posadas – Buenos Aires (AEP) 26/11/2026 21:45 – 23:25</t>
+          <t>Aerolíneas Argentinas AR 1812 Buenos Aires (AEP) – Puerto Madryn 16:00 – 18:05
+Aerolíneas Argentinas AR 1813 Puerto Madryn – Buenos Aires (AEP) 19:05 – 20:55</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>1 bolso de mano</t>
+          <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 1.323.740 (por persona en base doble — total con impuestos)
-Precio total por persona publicado por el operador en base a 2 adultos y 2 niños (incluye impuestos). La ficha no publica valor en base doble: se carga el publicado y se marca para revisión.</t>
+          <t>Desde ARS 676.299 (por persona en base doble — precio estimado, se cotiza al consultar)
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2419,12 +2421,12 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2027-07-31</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>categoría de algunos hoteles; itinerario día por día (la ficha no lo tiene)</t>
+          <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr"/>
@@ -2443,33 +2445,32 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Ushuaia &amp; El Calafate — 24 de noviembre 2026</t>
+          <t>Valle de la Luna con noche en Valle Fértil</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://cuartocontinente.com/es/idea/22204583/ushuaia-el-calafate?country=AR</t>
+          <t>https://cuartocontinente.com/es/idea/15448792/valle-de-la-luna-con-noche-en-valle-fertil?country=AR</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>24 de noviembre 2026</t>
+          <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Ushuaia: Hotel Rosa de los Vientos · 3 noches · Desayuno
-El Calafate: Kapenke Hotel · 3 noches · Desayuno</t>
+          <t>San Juan: America Apart Hotel · 2 noches · Desayuno buffet
+Valle Fértil: Hostería Valle Fértil · 1 noches · Media pensión</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Aerolíneas Argentinas AR 1876 Buenos Aires (AEP) – Ushuaia 24/11/2026 05:05 – 08:45
-Aerolíneas Argentinas AR 1895 Ushuaia – El Calafate 27/11/2026 09:20 – 10:40
-Aerolíneas Argentinas AR 1899 El Calafate – Buenos Aires (AEP) 30/11/2026 18:40 – 21:40</t>
+          <t>Aerolíneas Argentinas AR 1444 Buenos Aires (AEP) – San Juan 07:45 – 09:45
+Aerolíneas Argentinas AR 1445 San Juan – Buenos Aires (AEP) 10:30 – 12:10</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2479,8 +2480,9 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 1.342.389 (por persona en base doble — total con impuestos)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes.</t>
+          <t>Desde ARS 1.395.002 (por persona en base single — precio estimado, se cotiza al consultar)
+Precio total por persona publicado por el operador para 1 adulto (incluye impuestos), fecha de ejemplo 17–20 nov 2026. Salidas diarias: la ficha no da fecha límite, se carga vigencia 31/12/2026 para revisión. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).
+single: ARS 1.395.002</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2490,12 +2492,12 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>2026-11-24</t>
+          <t>2027-07-31</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>categoría de algunos hoteles; itinerario día por día (la ficha no lo tiene)</t>
+          <t>categoría de algunos hoteles; fecha/horario de vuelos; precio en base doble (la ficha publica otra base)</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr"/>
@@ -2514,116 +2516,94 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Valle de la Luna con noche en Valle Fértil — Salidas diarias</t>
+          <t>Salta &amp; Purmamarca</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://cuartocontinente.com/es/idea/15448792/valle-de-la-luna-con-noche-en-valle-fertil?country=AR</t>
+          <t>https://cuartocontinente.com/es/idea/25105671/salta-purmamarca-ida-y-vuelta-desde-salta?country=AR</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Salidas diarias (ejemplo: 17 de noviembre 2026)</t>
+          <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>San Juan: America Apart Hotel · 2 noches · Desayuno buffet
-Valle Fértil: Hostería Valle Fértil · 1 noches · Media pensión</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Aerolíneas Argentinas AR 1444 Buenos Aires (AEP) – San Juan 17/11/2026 07:45 – 09:45
-Aerolíneas Argentinas AR 1445 San Juan – Buenos Aires (AEP) 20/11/2026 10:30 – 12:10</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>1 valija en bodega (1 PC) + equipaje de mano</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>Desde ARS 1.395.002 (por persona en base single — total con impuestos)
-Precio total por persona publicado por el operador para 1 adulto (incluye impuestos), fecha de ejemplo 17–20 nov 2026. Salidas diarias: la ficha no da fecha límite, se carga vigencia 31/12/2026 para revisión.
-single: ARS 1.395.002</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>categoría de algunos hoteles; precio en base doble (la ficha publica otra base)</t>
-        </is>
-      </c>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>NUEVO</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Salta &amp; Purmamarca — 12 de abril 2027</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>https://cuartocontinente.com/es/idea/25105671/salta-purmamarca-ida-y-vuelta-desde-salta?country=AR</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>12 de abril 2027</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>Salta: Roomie Salta by DOT · 2 noches · Desayuno
 Purmamarca: El Refugio de Coquena · 2 noches · Desayuno
 Salta: Hotel del Tren · 1 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Aerolíneas Argentinas AR 1498 Buenos Aires (AEP) – Salta 12/04/2027 14:40 – 16:55
-Aerolíneas Argentinas AR 1489 Salta – Buenos Aires (AEP) 17/04/2027 07:55 – 10:00</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Aerolíneas Argentinas AR 1498 Buenos Aires (AEP) – Salta 14:40 – 16:55
+Aerolíneas Argentinas AR 1489 Salta – Buenos Aires (AEP) 07:55 – 10:00</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Desde ARS 1.362.212 (por persona en base single — precio estimado, se cotiza al consultar)
+Precio total por persona publicado por el operador para 1 adulto (incluye impuestos); no publica base doble. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).
+single: ARS 1.362.212</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>2027-07-31</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>categoría de algunos hoteles; fecha/horario de vuelos; precio en base doble (la ficha publica otra base)</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ELIMINADO (pedido del 15/10/2026)</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Esteros del Iberá</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>https://cuartocontinente.com/es/idea/64460563/esteros-del-ibera?country=AR</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Desde ARS 1.362.212 (por persona en base single — total con impuestos)
-Precio total por persona publicado por el operador para 1 adulto (incluye impuestos); no publica base doble.
-single: ARS 1.362.212</t>
+          <t>ARS 1.323.740 (2 adultos + 2 niños)</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2631,14 +2611,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>2027-04-12</t>
-        </is>
-      </c>
+      <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>categoría de algunos hoteles; precio en base doble (la ficha publica otra base)</t>
+          <t>eliminado del sitio: sin precio por persona base doble</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Parte 6f: Cuarto Continente con vigencia a 30 días (14/11/2026); Mágicamente Europa (JT-2193) vuelve a USD 4.622 con tasas hoteleras dentro del Desde; regiones_extra para listados: egipto-jordania aparece también en /medio-oriente/
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -1992,8 +1992,8 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Desde USD 4.526 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
-Tarifa USD 3.696 + impuestos aéreos USD 582 + IVA y gastos USD 248 = USD 4.526 (como publica la ficha). Tasas hoteleras obligatorias USD 94 + USD 2 de gastos aparte, se pagan al reservar. Triple y single: consultar. Seña USD 2.100.</t>
+          <t>Desde USD 4.622 (por persona en base doble — tarifa + impuestos + IVA/gastos + tasas hoteleras obligatorias)
+Tarifa USD 3.696 + impuestos aéreos USD 582 + IVA y gastos USD 248 + tasas hoteleras obligatorias USD 94 + gastos USD 2 = USD 4.622 (la ficha publica 4.526 y las tasas aparte; por regla, todo cargo obligatorio que se paga al reservar va dentro del Desde). Triple y single: consultar. Seña USD 2.100.</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2062,7 +2062,7 @@
       <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 567.676 (por persona en base doble — precio estimado, se cotiza al consultar)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>2027-07-31</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -2081,7 +2081,11 @@
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2131,7 +2135,7 @@
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 949.630 (por persona en base doble — precio estimado, se cotiza al consultar)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2141,7 +2145,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>2027-07-31</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -2150,7 +2154,11 @@
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2200,7 +2208,7 @@
       <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 651.624 (por persona en base doble — precio estimado, se cotiza al consultar)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2210,7 +2218,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>2027-07-31</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -2219,7 +2227,11 @@
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2271,7 +2283,7 @@
       <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 1.280.826 (por persona en base doble — precio estimado, se cotiza al consultar)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2281,7 +2293,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2027-07-31</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -2290,7 +2302,11 @@
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2342,7 +2358,7 @@
       <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 1.342.389 (por persona en base doble — precio estimado, se cotiza al consultar)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2352,7 +2368,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>2027-07-31</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2361,7 +2377,11 @@
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2411,7 +2431,7 @@
       <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 676.299 (por persona en base doble — precio estimado, se cotiza al consultar)
-Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).</t>
+Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2421,7 +2441,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>2027-07-31</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2430,7 +2450,11 @@
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2481,7 +2505,7 @@
       <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 1.395.002 (por persona en base single — precio estimado, se cotiza al consultar)
-Precio total por persona publicado por el operador para 1 adulto (incluye impuestos), fecha de ejemplo 17–20 nov 2026. Salidas diarias: la ficha no da fecha límite, se carga vigencia 31/12/2026 para revisión. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).
+Precio total por persona publicado por el operador para 1 adulto (incluye impuestos), fecha de ejemplo 17–20 nov 2026. Salidas diarias: la ficha no da fecha límite, se carga vigencia 31/12/2026 para revisión. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.
 single: ARS 1.395.002</t>
         </is>
       </c>
@@ -2492,7 +2516,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>2027-07-31</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2501,7 +2525,11 @@
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2553,7 +2581,7 @@
       <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 1.362.212 (por persona en base single — precio estimado, se cotiza al consultar)
-Precio total por persona publicado por el operador para 1 adulto (incluye impuestos); no publica base doble. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario).
+Precio total por persona publicado por el operador para 1 adulto (incluye impuestos); no publica base doble. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.
 single: ARS 1.362.212</t>
         </is>
       </c>
@@ -2564,7 +2592,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>2027-07-31</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -2573,7 +2601,11 @@
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Código de referencia interno: codigo_ref en los 57 paquetes activos (KM/JT/CC/PI/AS por URL de la ficha, GEA para los del portal anterior), 'Cód. …' chiquito bajo el precio del detalle, paquete_codigo en el dataLayer y data-paquete-codigo en los botones de WhatsApp; columna Código en la planilla; design.css v12
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisión parte 6" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Revisión parte 6'!$A$1:$O$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Revisión parte 6'!$A$1:$P$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,24 +430,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,60 +469,65 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>URL ficha</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Salidas</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Noches</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Hoteles</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Vuelos</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Equipaje</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Precio desde y desglose</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Moneda</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Vigencia</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Faltantes</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>OK / Corrección</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Comentario</t>
         </is>
@@ -545,18 +551,23 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>KM-1145</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/1145/India-&amp;-Maldivas%C2%A0</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>20 de enero 2027</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Delhi: The Lalit Hotel · 3 noches · Desayuno
 Mandawa: Vivaana Museum · 1 noches · Desayuno
@@ -567,7 +578,7 @@
 Maldivas: Centara Ras Fushi · 4 noches · All Inclusive</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Turkish Airlines TK 016 Buenos Aires (EZE) – Estambul 20/01/2027 23:55 – 22:35 (+1)
 Turkish Airlines TK 716 Estambul – Delhi 22/01/2027 20:50 – 05:20 (+1)
@@ -575,35 +586,35 @@
 Turkish Airlines TK 015 Estambul – Buenos Aires (EZE) 08/02/2027 10:00 – 22:25</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Desde USD 9.440 (por persona en base doble — total con impuestos)
 Base doble USD 7.750 + impuestos USD 1.690 (DNT, IVA, gastos y propinas) = USD 9.440. Single: 7.750 + 2.950 + 1.690 = 12.390. Triple igual a doble según ficha.
 triple: USD 9.440 · single: USD 12.390</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>2027-01-20</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; equipaje</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -623,18 +634,23 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>KM-1147</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/1147/Sudafrica%C2%A0&amp;-Mauritius</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>8 de febrero 2027 — South African Airways vía San Pablo</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Johannesburgo: Silverbirch Hotel 4* · 1 noches · Desayuno
 Área Kruger: Moditlo / Shidlulli, reserva privada Karongwe · 2 noches · Pensión completa
@@ -642,7 +658,7 @@
 Ciudad del Cabo: Southern Sun Waterfront 4* · 4 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Gol G3 7681 Buenos Aires (AEP) – San Pablo (GRU)
 South African Airways SA 223 San Pablo – Johannesburgo
@@ -652,35 +668,35 @@
 Gol G3 7648 San Pablo – Buenos Aires (AEP)</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Desde USD 9.820 (por persona en base doble — total con impuestos)
 Base doble USD 7.950 + impuestos USD 1.870 (DNT, IVA, gastos y propinas) = USD 9.820. Single: 7.950 + 2.880 + 1.870 = 12.700. Los vuelos de la ficha figuran con fechas de noviembre (16NOV–28NOV): se cargan solo aerolínea, ruta y número. Decisión del usuario (15/10/2026): se publica la salida del 8 de febrero 2027.
 single: USD 12.700</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>2027-02-08</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos; equipaje</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -700,18 +716,23 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>KM-4</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/4/Kenia-&amp;Tanzania</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>22 de febrero 2027</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Nairobi: Sarova Stanley Hotel 4* · 2 noches · Desayuno
 Lago Nakuru: Sarova Lion Hill Game Lodge 4* · 1 noches · Pensión completa
@@ -722,7 +743,7 @@
 Zanzíbar: Riu Jambo Zanzibar 4* · 4 noches · All Inclusive</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Ethiopian Airlines ET 507 Buenos Aires (EZE) – Addis Abeba 22/02/2027 21:30 – 19:30 (+1)
 Ethiopian Airlines ET 308 Addis Abeba – Nairobi 23/02/2027 23:35 – 01:40 (+1)
@@ -730,35 +751,35 @@
 Ethiopian Airlines ET 506 Addis Abeba – Buenos Aires (EZE) 10/03/2027 09:50 – 19:55</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Desde USD 11.900 (por persona en base doble — total con impuestos)
 Base doble USD 9.980 + impuestos USD 1.920 (visa de Kenia, DNT, IVA, gastos y propinas) = USD 11.900. Single: 9.980 + 1.850 + 1.920 = 13.750.
 single: USD 13.750</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>2027-02-22</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>equipaje</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -778,18 +799,23 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>KM-1115</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/1115/Vietnam,-Camboya-&amp;-Tailandia-2027</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>7 de marzo 2027</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Hanoi: Grand Mercure 4* · 2 noches · Desayuno
 Bahía de Lan Ha: Indochine Premium Ha Long (crucero) 4* · 1 noches · Pensión completa
@@ -801,7 +827,7 @@
 Phuket: Pullman Phuket Panwa Beach 4* · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Turkish Airlines TK 016 Buenos Aires (EZE) – Estambul 07/03/2027 23:55 – 22:35 (+1)
 Turkish Airlines TK 164 Estambul – Hanoi 09/03/2027 02:25 – 15:25
@@ -809,35 +835,35 @@
 Turkish Airlines TK 015 Estambul – Buenos Aires (EZE) 26/03/2027 10:00 – 22:25</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Desde USD 9.740 (por persona en base doble — total con impuestos)
 Base doble USD 7.950 + impuestos USD 1.790 (IVA, gastos, DNT, tasas y propinas) = USD 9.740. Single: 7.950 + 2.280 + 1.790 = 12.020. Reemplaza la versión de noviembre 2026 (26 días, USD 14.330).
 single: USD 12.020</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>2027-03-07</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>equipaje</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -857,18 +883,23 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>KM-1116</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/1116/Fiesta-%22Holi%22---India-2027</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>14 de marzo 2027</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Delhi: The Lalit Hotel 5* · 3 noches · Desayuno
 Agra: Grand Mercure 4* · 2 noches · Desayuno
@@ -881,7 +912,7 @@
 Mumbai: ITC Grand Central 4* Sup · 2 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Ethiopian Airlines ET 507 Buenos Aires (EZE) – Addis Abeba 14/03/2027 21:30 – 19:30 (+1)
 Ethiopian Airlines ET 686 Addis Abeba – Delhi 15/03/2027 23:10 – 08:05 (+1)
@@ -889,35 +920,35 @@
 Ethiopian Airlines ET 506 Addis Abeba – Buenos Aires (EZE) 02/04/2027 09:50 – 20:25</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Desde USD 7.890 (por persona en base doble — total con impuestos)
 Base doble USD 6.350 + impuestos USD 1.540 (DNT, IVA, gastos y propinas) = USD 7.890. Single: 6.350 + 1.850 + 1.540 = 9.740.
 single: USD 9.740</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>2027-03-14</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; equipaje</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -937,18 +968,23 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>KM-1117</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/1117/Egipto-&amp;-Jordania%C2%A0</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>17 de marzo 2027</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>El Cairo: Sofitel Cairo Downtown 4* · 5 noches
 Crucero Nilo: Blue Shadow / Opera 4* · 4 noches
@@ -958,7 +994,7 @@
 Mar Muerto: Holiday Inn Dead Sea 4* · 2 noches</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Ethiopian Airlines ET 507 Buenos Aires (EZE) – Addis Abeba 17/03/2027 21:30 – 19:30 (+1)
 Ethiopian Airlines ET 452 Addis Abeba – El Cairo 18/03/2027 22:05 – 01:05 (+1)
@@ -966,35 +1002,35 @@
 Ethiopian Airlines ET 506 Addis Abeba – Buenos Aires (EZE) 02/04/2027 09:50 – 20:25</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Desde USD 8.420 (por persona en base doble — total con impuestos)
 Base doble USD 6.580 + impuestos USD 1.840 (DNT, IVA, gastos, visa de Egipto y propinas) = USD 8.420 (sin cambios). Single: 6.580 + 2.650 + 1.840 = 11.070.
 single: USD 11.070</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>2027-03-17</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; equipaje</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1014,18 +1050,23 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>KM-1090</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/1090/Corea-&amp;-Jap%C3%B3n---%22Cherry-Blossom%22</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>17 de marzo 2027</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Seúl: Nine Tree Parnas Myeongdong II 4* · 3 noches · Desayuno
 Gyeongju: Gyeongju Kolon Hotel 4* · 2 noches · Desayuno
@@ -1038,7 +1079,7 @@
 Tokio: Hotel New Otani 4* · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Turkish Airlines TK 016 Buenos Aires (EZE) – Estambul 17/03/2027 23:55 – 22:35 (+1)
 Turkish Airlines TK 090 Estambul – Seúl (Incheon) 19/03/2027 02:15 – 18:20
@@ -1046,35 +1087,35 @@
 Turkish Airlines TK 015 Estambul – Buenos Aires (EZE) 07/04/2027 10:35 – 22:25</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Desde USD 14.810 (por persona en base doble — total con impuestos)
 Base doble USD 12.880 + impuestos USD 1.930 (DNT, IVA, gastos y propinas) = USD 14.810. Single: 12.880 + 4.170 + 1.930 = 18.980.
 single: USD 18.980</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>2027-03-17</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; equipaje</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1094,18 +1135,23 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>KM-2</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/2/China&amp;-T%C3%ADbet</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>6 de abril 2027</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Beijing: Kerry Hotel Beijing 5* · 4 noches · Desayuno
 Xi'an: Hilton Xian High-tech Zone 5* · 2 noches · Desayuno
@@ -1117,7 +1163,7 @@
 Shanghái: Hengshan Garden Hotel 5* · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Turkish Airlines TK 016 Buenos Aires (EZE) – Estambul 06/04/2027 23:55 – 22:45 (+1)
 Turkish Airlines TK 088 Estambul – Beijing 08/04/2027 01:40 – 15:35
@@ -1125,35 +1171,35 @@
 Turkish Airlines TK 015 Estambul – Buenos Aires (EZE) 28/04/2027 10:35 – 22:25</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Desde USD 10.220 (por persona en base doble — total con impuestos)
 Base doble USD 8.350 + impuestos USD 1.870 (DNT, IVA, visa de China, gastos y propinas) = USD 10.220. Single: 8.350 + 1.920 + 1.870 = 12.140.
 single: USD 12.140</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>2027-04-06</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>equipaje</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1173,18 +1219,23 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>KM-1126</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/1126/Hong-Kong-&amp;-China-2027</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>10 de mayo 2027</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Hong Kong: Royal Garden Hotel 4* Sup · 2 noches · Desayuno
 Beijing: Kerry Hotel 5* · 4 noches · Desayuno
@@ -1195,7 +1246,7 @@
 Shanghái: Renaissance Shanghai Zhongshan Park 5* · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Turkish Airlines TK 016 Buenos Aires (EZE) – Estambul 10/05/2027 23:55 – 22:45 (+1)
 Turkish Airlines TK 070 Estambul – Hong Kong 12/05/2027 01:35 – 17:20
@@ -1203,35 +1254,35 @@
 Turkish Airlines TK 015 Estambul – Buenos Aires (EZE) 30/05/2027 10:35 – 22:25</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Desde USD 8.230 (por persona en base doble — total con impuestos)
 Base doble USD 6.680 + impuestos USD 1.550 (DNT, IVA, gastos y propinas) = USD 8.230. Single: 6.680 + 1.750 + 1.550 = 9.980.
 single: USD 9.980</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>2027-05-10</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>equipaje</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1251,18 +1302,23 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>KM-1146</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>https://www.kingmidas.com.ar/itinerario/1146/Malasia,-Singapur-&amp;-Bali</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>24 de mayo 2027</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Kuala Lumpur: Capri by Fraser Bukit Bintang 4* · 3 noches · Desayuno
 Malaca: Swiss Garden Melaka 4* · 1 noches · Desayuno
@@ -1271,7 +1327,7 @@
 Nusa Dua: Merusaka Nusa Dua 4* · 5 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Turkish Airlines TK 016 Buenos Aires (EZE) – Estambul 24/05/2027 23:55 – 22:45 (+1)
 Turkish Airlines TK 060 Estambul – Kuala Lumpur 26/05/2027 01:40 – 17:15
@@ -1279,35 +1335,35 @@
 Turkish Airlines TK 015 Estambul – Buenos Aires (EZE) 12/06/2027 10:35 – 22:25</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>no figura en la ficha</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Desde USD 9.435 (por persona en base doble — total con impuestos)
 Base doble USD 7.820 + impuestos USD 1.615 (DNT, IVA, gastos y propinas) = USD 9.435. Single: 7.820 + 2.480 + 1.615 = 11.915.
 single: USD 11.915</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>2027-05-24</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>equipaje</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1327,18 +1383,23 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>JT-2187</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.com.ar/micrositio.php?id=2187</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>23 de abril 2027</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Madrid: Chamartín The One 4* · 2 noches · Desayuno
 Burdeos: Mercure Bordeaux Le Lac 4* · 2 noches · Desayuno
@@ -1348,41 +1409,41 @@
 Ámsterdam: Park Plaza Amsterdam Airport · 2 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 23/04/2027 17:50 – 10:45 (+1)
 Iberia IB 107 Madrid – Buenos Aires (EZE) 10/05/2027 12:15 – 19:55</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Desde USD 5.024 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
 Tarifa USD 4.160 + impuestos aéreos USD 584 + IVA y gastos USD 280 = USD 5.024. Triple USD 4.946. Single USD 6.892. Seña USD 2.300.
 triple: USD 4.946 · single: USD 6.892</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>2027-01-15</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1402,18 +1463,23 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>JT-2143</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.tur.ar/micrositio.php?id=2143</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>21 de mayo 2027</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Madrid: Praga 4* · 2 noches · Desayuno
 Barcelona: AC Som 4* · 1 noches · Desayuno
@@ -1426,41 +1492,41 @@
 Burdeos: Mercure Bordeaux Centre Meriadeck 3* · 1 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 21/05/2027 17:50 – 10:45 (+1)
 Iberia IB 105 Madrid – Buenos Aires (EZE) 07/06/2027 08:45 – 16:25</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Desde USD 4.858 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
 Tarifa USD 4.006 + impuestos aéreos USD 583 + IVA y gastos USD 269 = USD 4.858. Triple USD 4.782. Single USD 6.445. Seña USD 2.200.
 triple: USD 4.782 · single: USD 6.445</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>2027-01-15</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1480,18 +1546,23 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>JT-2149</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.com.ar/micrositio.php?id=2149</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>2 de mayo 2027</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Madrid: Chamartín The One / Praga 4* · 5 noches · Desayuno
 Burdeos: Mercure Bordeaux Le Lac 4* · 1 noches · Desayuno
@@ -1504,41 +1575,41 @@
 Barcelona: Front Air Congress 4* · 1 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 02/05/2027 17:50 – 10:55 (+1)
 Iberia IB 107 Madrid – Buenos Aires (EZE) 20/05/2027 12:15 – 19:55</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Desde USD 4.554 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
 Tarifa USD 3.722 + impuestos aéreos USD 581 + IVA y gastos USD 251 = USD 4.554. Triple USD 4.484. Single USD 6.077.
 triple: USD 4.484 · single: USD 6.077</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>2027-01-15</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1558,18 +1629,23 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>JT-2160</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.com.ar/micrositio.php?id=2160</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>16 de abril 2027</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Madrid: Praga 4* · 3 noches · Desayuno
 Granada: Saray 4* · 1 noches · Desayuno
@@ -1583,41 +1659,41 @@
 Lisboa: VIP Executive Entrecampos 4* · 2 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 16/04/2027 17:50 – 10:45 (+1)
 Iberia IB 107 Madrid – Buenos Aires (EZE) 03/05/2027 12:15 – 19:55</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Desde USD 4.710 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
 Tarifa USD 3.867 + impuestos aéreos USD 582 + IVA y gastos USD 261 = USD 4.710. Triple USD 4.636. Single USD 6.067. Seña USD 2.300.
 triple: USD 4.636 · single: USD 6.067</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>2027-01-15</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1637,18 +1713,23 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>JT-2181</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.com.ar/micrositio.php?id=2181</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>7 de mayo 2027</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Madrid: Praga 4* · 3 noches · Desayuno
 Granada: Macia Condor 4* · 1 noches · Desayuno
@@ -1663,41 +1744,41 @@
 Valencia: DWO Valencia 4* · 1 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 07/05/2027 17:50 – 10:45 (+1)
 Iberia IB 105 Madrid – Buenos Aires (EZE) 24/05/2027 08:45 – 16:25</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Desde USD 4.723 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
 Tarifa USD 3.880 + impuestos aéreos USD 583 + IVA y gastos USD 260 = USD 4.723. Triple USD 4.651. Single USD 6.195. Seña USD 2.250.
 triple: USD 4.651 · single: USD 6.195</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>2027-01-15</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1717,18 +1798,23 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>JT-2205</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.com.ar/micrositio.php?id=2205</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>6 de junio 2027</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Madrid: Praga 4* · 4 noches · Desayuno
 Granada: Saray 4* · 1 noches · Desayuno
@@ -1743,41 +1829,41 @@
 Lourdes: Alba 4* · 2 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 06/06/2027 17:50 – 10:45 (+1)
 Iberia IB 107 Madrid – Buenos Aires (EZE) 24/06/2027 12:15 – 19:55</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Desde USD 4.885 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
 Tarifa USD 4.031 + impuestos aéreos USD 581 + IVA y gastos USD 273 = USD 4.885. Triple USD 4.807. Single USD 6.489. Seña USD 2.200.
 triple: USD 4.807 · single: USD 6.489</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>2027-01-15</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1797,18 +1883,23 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>JT-2156</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.com.ar/micrositio.php?id=2156</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>9 de mayo 2027</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Madrid: Gran Versalles 4* · 3 noches · Desayuno
 Burdeos: Ibis Styles Bordeaux Centre Meriadeck 3* · 1 noches · Desayuno
@@ -1822,41 +1913,41 @@
 Barcelona: Barcelona 505 4* · 2 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 09/05/2027 17:50 – 10:45 (+1)
 Iberia IB 105 Madrid – Buenos Aires (EZE) 27/05/2027 08:45 – 16:25</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Desde USD 5.679 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
 Tarifa USD 4.772 + impuestos aéreos USD 581 + IVA y gastos USD 326 = USD 5.679. Triple USD 5.607. Single USD 7.520. Seña USD 2.300.
 triple: USD 5.607 · single: USD 7.520</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>2027-01-15</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1876,18 +1967,23 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>JT-2253</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.com.ar/micrositio.php?id=2253</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>4 de abril 2027</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Madrid: Chamartín The One 4* · 5 noches · Desayuno
 Burdeos: Ibis Styles Bordeaux Gare Saint-Jean 3* · 1 noches · Desayuno
@@ -1900,41 +1996,41 @@
 Barcelona: Catalonia Barcelona Plaza 4* · 1 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 04/04/2027 17:50 – 10:45 (+1)
 Iberia IB 107 Madrid – Buenos Aires (EZE) 22/04/2027 12:15 – 19:55</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Desde USD 5.187 (por persona en base doble — tarifa + impuestos aéreos + IVA y gastos)
 Tarifa USD 4.313 + impuestos aéreos USD 581 + IVA y gastos USD 293 = USD 5.187. Triple USD 5.052. Single USD 6.619. Seña USD 2.200.
 triple: USD 5.052 · single: USD 6.619</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>2027-04-04</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1954,18 +2050,23 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
+          <t>JT-2193</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
           <t>https://www.juliatours.com.ar/micrositio.php?id=2193</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>9 de abril 2027</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Madrid: Hampton by Hilton Alcobendas 3* · 3 noches · Desayuno
 Burdeos: B&amp;B Hotel Bordeaux Bègles 3* · 1 noches · Desayuno
@@ -1979,40 +2080,40 @@
 Barcelona: Frontair Congress 4* · 1 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Iberia IB 106 Buenos Aires (EZE) – Madrid 09/04/2027 17:50 – 10:45 (+1)
 Iberia IB 107 Madrid – Buenos Aires (EZE) 26/04/2027 12:15 – 19:55</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>1 valija de hasta 23 kg por persona en todo el recorrido</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Desde USD 4.622 (por persona en base doble — tarifa + impuestos + IVA/gastos + tasas hoteleras obligatorias)
 Tarifa USD 3.696 + impuestos aéreos USD 582 + IVA y gastos USD 248 + tasas hoteleras obligatorias USD 94 + gastos USD 2 = USD 4.622 (la ficha publica 4.526 y las tasas aparte; por regla, todo cargo obligatorio que se paga al reservar va dentro del Desde). Triple y single: consultar. Seña USD 2.100.</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>2027-04-09</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>precio single/triple</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2032,56 +2133,61 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
+          <t>CC-22256231</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/22256231/escapada-a-mendoza?country=AR</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Mendoza: Hotel Cordón del Plata · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Aerolíneas Argentinas AR 1402 Buenos Aires (AEP) – Mendoza 07:40 – 09:40
 Aerolíneas Argentinas AR 1401 Mendoza – Buenos Aires (AEP) 07:30 – 09:10</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 567.676 (por persona en base doble — precio estimado, se cotiza al consultar)
 Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr">
         <is>
           <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
         </is>
@@ -2105,56 +2211,61 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
+          <t>CC-22203065</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/22203065/ushuaia?country=AR</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="G22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Ushuaia: Del Bosque Apart &amp; Hotel · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Aerolíneas Argentinas AR 1886 Buenos Aires (AEP) – Ushuaia 05:50 – 09:30
 Aerolíneas Argentinas AR 1871 Ushuaia – Buenos Aires (AEP) 08:20 – 11:50</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 949.630 (por persona en base doble — precio estimado, se cotiza al consultar)
 Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr">
         <is>
           <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
         </is>
@@ -2178,56 +2289,61 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
+          <t>CC-40420928</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/40420928/bariloche-lo-tiene-todo?country=AR</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Bariloche: Hotel Nevada · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Aerolíneas Argentinas AR 1680 Buenos Aires (AEP) – Bariloche 04:35 – 07:00
 Aerolíneas Argentinas AR 1681 Bariloche – Buenos Aires (AEP) 11:55 – 14:00</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 651.624 (por persona en base doble — precio estimado, se cotiza al consultar)
 Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
         </is>
@@ -2251,58 +2367,63 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
+          <t>CC-24058473</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/24058473/vuelta-al-norte-argentino?country=AR</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="G24" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>San Miguel de Tucumán: Hotel Francia · 1 noches · Desayuno continental
 Cafayate: Hotel Asturias · 1 noches · Desayuno
 Salta: Altos de Balcarce · 4 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Aerolíneas Argentinas AR 1468 Buenos Aires (AEP) – Tucumán 04:55 – 06:55
 Aerolíneas Argentinas AR 1489 Salta – Buenos Aires (AEP) 08:05 – 10:10</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 1.280.826 (por persona en base doble — precio estimado, se cotiza al consultar)
 Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr">
         <is>
           <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
         </is>
@@ -2326,58 +2447,63 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
+          <t>CC-22204583</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/22204583/ushuaia-el-calafate?country=AR</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="G25" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Ushuaia: Hotel Rosa de los Vientos · 3 noches · Desayuno
 El Calafate: Kapenke Hotel · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Aerolíneas Argentinas AR 1876 Buenos Aires (AEP) – Ushuaia 05:05 – 08:45
 Aerolíneas Argentinas AR 1895 Ushuaia – El Calafate 09:20 – 10:40
 Aerolíneas Argentinas AR 1899 El Calafate – Buenos Aires (AEP) 18:40 – 21:40</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 1.342.389 (por persona en base doble — precio estimado, se cotiza al consultar)
 Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr">
         <is>
           <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
         </is>
@@ -2401,56 +2527,61 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
+          <t>CC-37028317</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/37028317/puerto-madryn?country=AR</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Puerto Madryn: Parry Hotel · 3 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Aerolíneas Argentinas AR 1812 Buenos Aires (AEP) – Puerto Madryn 16:00 – 18:05
 Aerolíneas Argentinas AR 1813 Puerto Madryn – Buenos Aires (AEP) 19:05 – 20:55</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 676.299 (por persona en base doble — precio estimado, se cotiza al consultar)
 Precio total por persona publicado por el operador en base a 2 adultos (incluye impuestos); la ficha no desglosa componentes. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr">
         <is>
           <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
         </is>
@@ -2474,58 +2605,63 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
+          <t>CC-15448792</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/15448792/valle-de-la-luna-con-noche-en-valle-fertil?country=AR</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="G27" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>San Juan: America Apart Hotel · 2 noches · Desayuno buffet
 Valle Fértil: Hostería Valle Fértil · 1 noches · Media pensión</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Aerolíneas Argentinas AR 1444 Buenos Aires (AEP) – San Juan 07:45 – 09:45
 Aerolíneas Argentinas AR 1445 San Juan – Buenos Aires (AEP) 10:30 – 12:10</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 1.395.002 (por persona en base single — precio estimado, se cotiza al consultar)
 Precio total por persona publicado por el operador para 1 adulto (incluye impuestos), fecha de ejemplo 17–20 nov 2026. Salidas diarias: la ficha no da fecha límite, se carga vigencia 31/12/2026 para revisión. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.
 single: ARS 1.395.002</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos; precio en base doble (la ficha publica otra base)</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
         </is>
@@ -2549,59 +2685,64 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
+          <t>CC-25105671</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/25105671/salta-purmamarca-ida-y-vuelta-desde-salta?country=AR</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Fecha a elección, hasta julio 2027</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Salta: Roomie Salta by DOT · 2 noches · Desayuno
 Purmamarca: El Refugio de Coquena · 2 noches · Desayuno
 Salta: Hotel del Tren · 1 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>Aerolíneas Argentinas AR 1498 Buenos Aires (AEP) – Salta 14:40 – 16:55
 Aerolíneas Argentinas AR 1489 Salta – Buenos Aires (AEP) 07:55 – 10:00</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>1 valija en bodega (1 PC) + equipaje de mano</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Desde ARS 1.362.212 (por persona en base single — precio estimado, se cotiza al consultar)
 Precio total por persona publicado por el operador para 1 adulto (incluye impuestos); no publica base doble. Cotización de referencia del 15/10/2026 para una fecha puntual: se publica como precio estimado 'Desde' sin fecha fija, viajable hasta julio 2027 (indicación del usuario). Vigencia 30 días (hasta 14/11/2026): precio en ARS de referencia, actualizar cada 30 días.
 single: ARS 1.362.212</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; fecha/horario de vuelos; precio en base doble (la ficha publica otra base)</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr">
         <is>
           <t>Precio en ARS de referencia: actualizar cada 30 días o se baja solo</t>
         </is>
@@ -2625,32 +2766,37 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
+          <t>CC-64460563</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/64460563/esteros-del-ibera?country=AR</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>ARS 1.323.740 (2 adultos + 2 niños)</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>eliminado del sitio: sin precio por persona base doble</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2670,36 +2816,41 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
+          <t>CC-14446258</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/14446258/salta-con-cafayate</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>10–13 jun 2026 (pasada)</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>ARS 499.072</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>sin salidas futuras: no se carga</t>
         </is>
       </c>
-      <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2719,28 +2870,33 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
+          <t>CC-22668768</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/22668768/mendoza-san-rafael</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>14–20 jun 2026 (pasada)</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>sin salidas futuras: no se carga</t>
         </is>
       </c>
-      <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2760,28 +2916,33 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
+          <t>CC-34918244</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/34918244/bariloche-villa-la-angostura-san-martin-de-los-andes</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>10–19 jun 2026 (pasada)</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>sin salidas futuras: no se carga</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2801,28 +2962,33 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
+          <t>CC-22365887</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
           <t>https://cuartocontinente.com/es/idea/22365887/el-calafate-chalten-ushuaia</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>25 mar – 2 abr 2026 (pasada)</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>sin salidas futuras: no se carga</t>
         </is>
       </c>
-      <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2842,56 +3008,61 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
+          <t>PI-65533521</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
           <t>https://piamonte.com/es/idea/65533521/miches-04-01-verano-2027</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>4 de enero 2027</t>
         </is>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="G34" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Miches: Viva Miches by Wyndham, A Trademark Resort · 12 noches · Todo Incluido</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>LATAM Buenos Aires – Punta Cana (1 escala) 04/01/2027 07:45 – 17:35
 LATAM Punta Cana – Buenos Aires (1 escala) 16/01/2027 19:35 – 07:40 (+1)</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>1 artículo personal (10 kg) + 1 carry on (10 kg) + 1 valija en bodega de 23 kg</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Desde USD 3.744 (por persona en base doble — total con impuestos)
 Precio total por persona en base doble publicado por el operador (incluye IVA, DNT, impuestos y gastos administrativos); la ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>2027-01-04</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; número de algunos vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2911,56 +3082,61 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
+          <t>PI-51938153</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
           <t>https://piamonte.com/es/idea/51938153/caribe-con-crucero-07-01-cabina-externa</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>7 de enero 2027</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="G35" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Punta Cana (Uvero Alto): Ocean El Faro · 3 noches · Todo Incluido</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>Arajet DM 6265 Buenos Aires – Punta Cana (directo) 07/01/2027 11:00 – 17:55
 Arajet DM 6268 Punta Cana – Buenos Aires (directo) 17/01/2027 20:02 – 05:00 (+1)</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>1 artículo personal (6 kg) + 1 valija en bodega de 23 kg + selección de asiento</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Desde USD 3.293 (por persona en base doble — total con impuestos)
 Precio total por persona en base doble publicado por el operador (incluye IVA, DNT, impuestos y gastos administrativos); la ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>2027-01-07</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2980,56 +3156,61 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
+          <t>PI-52302197</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
           <t>https://piamonte.com/es/idea/52302197/aruba-09-01-verano-2027</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>9 de enero 2027</t>
         </is>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Palm Beach: TRYP by Wyndham Aruba Adults Only · 8 noches · Solo habitación</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>LATAM Buenos Aires – Aruba (1 escala) 09/01/2027 08:40 – 18:00
 LATAM Aruba – Buenos Aires (1 escala) 17/01/2027 19:10 – 06:20 (+1)</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>1 artículo personal (10 kg) + 1 carry on (10 kg) + 1 valija en bodega de 23 kg</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Desde USD 3.134 (por persona en base doble — total con impuestos)
 Precio total por persona en base doble publicado por el operador (incluye IVA, DNT, impuestos y gastos administrativos); la ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>2027-01-09</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; número de algunos vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3049,56 +3230,61 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
+          <t>PI-52975881</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
           <t>https://piamonte.com/es/idea/52975881/punta-cana-13-01-verano-2027</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>13 de enero 2027</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Punta Cana (Bávaro): Occidental Caribe · 10 noches · Todo Incluido</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>LATAM Buenos Aires – Punta Cana (1 escala) 13/01/2027 07:45 – 18:30
 LATAM Punta Cana – Buenos Aires (1 escala) 23/01/2027 19:35 – 07:40 (+1)</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>1 artículo personal (10 kg) + 1 carry on (10 kg) + 1 valija en bodega de 23 kg</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>Desde USD 2.988 (por persona en base doble — total con impuestos)
 Precio total por persona en base doble publicado por el operador (incluye IVA, DNT, impuestos y gastos administrativos); la ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>2027-01-13</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; número de algunos vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr"/>
       <c r="O37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3118,56 +3304,61 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
+          <t>PI-54740316</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
           <t>https://piamonte.com/es/idea/54740316/riviera-maya-18-01-verano-2027</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>18 de enero 2027</t>
         </is>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="G38" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Puerto Aventuras: Catalonia Riviera Maya Resort and Spa · 7 noches · Todo Incluido</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>Arajet Buenos Aires – Cancún (1 escala) 18/01/2027 06:00 – 16:55
 Arajet Cancún – Buenos Aires (1 escala) 25/01/2027 17:36 – 07:40 (+1)</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>1 artículo personal + 1 valija en bodega de 23 kg (no incluye carry on)</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Desde USD 2.396 (por persona en base doble — total con impuestos)
 Precio total por persona en base doble publicado por el operador (incluye IVA, DNT, impuestos y gastos administrativos); la ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>2027-01-18</t>
         </is>
       </c>
-      <c r="M38" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; número de algunos vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3187,56 +3378,61 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
+          <t>PI-55903469</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>https://piamonte.com/es/idea/55903469/costa-mujeres-18-01-verano-2027</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>18 de enero 2027</t>
         </is>
       </c>
-      <c r="F39" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Costa Mujeres: Riu Dunamar · 7 noches · Todo Incluido</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>Arajet Buenos Aires – Cancún (1 escala) 18/01/2027 06:00 – 16:55
 Arajet Cancún – Buenos Aires (1 escala) 25/01/2027 17:36 – 07:40 (+1)</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>1 artículo personal + 1 valija en bodega de 23 kg (no incluye carry on)</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>Desde USD 2.586 (por persona en base doble — total con impuestos)
 Precio total por persona en base doble publicado por el operador (incluye IVA, DNT, impuestos y gastos administrativos); la ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>2027-01-18</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; número de algunos vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N39" s="2" t="inlineStr"/>
       <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3256,57 +3452,62 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
+          <t>PI-63139480</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
           <t>https://piamonte.com/es/idea/63139480/riviera-maya-cancun-25-01-verano-2027</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>25 de enero 2027</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n">
+      <c r="G40" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Playa del Carmen: Iberostar Waves Paraíso Beach · 8 noches · Todo Incluido
 Cancún: Iberostar Selection Cancún · 2 noches · Todo Incluido</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>LATAM Buenos Aires – Cancún (1 escala) 25/01/2027 07:20 – 17:40
 LATAM Cancún – Buenos Aires (1 escala) 04/02/2027 15:25 – 06:05 (+1)</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>1 artículo personal (10 kg) + 1 carry on (10 kg) + 1 valija en bodega de 23 kg</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Desde USD 3.159 (por persona en base doble — total con impuestos)
 Precio total por persona en base doble publicado por el operador (incluye IVA, DNT, impuestos y gastos administrativos); la ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>2027-01-25</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; número de algunos vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3326,58 +3527,63 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
+          <t>PI-66158100</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
           <t>https://piamonte.com/es/idea/66158100/miami-bayahibe-14-02</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>14 de febrero 2027</t>
         </is>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Miami Beach: Chesterfield Hotel &amp; Suites · 5 noches · Solo habitación
 Bayahíbe: Catalonia Bayahibe · 5 noches · Todo Incluido</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>LATAM LA 542 Buenos Aires – Miami (directo) 14/02/2027 13:10 – 19:45
 LATAM LA 591 Miami – Punta Cana (directo) 19/02/2027 09:00 – 12:25
 LATAM Punta Cana – Buenos Aires (1 escala) 24/02/2027 18:40 – 06:05 (+1)</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>1 artículo personal (10 kg) + 1 carry on (10 kg) + 1 valija en bodega de 23 kg</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>Desde USD 3.485 (por persona en base doble — total con impuestos)
 Precio total por persona en base doble publicado por el operador (incluye IVA, DNT, impuestos y gastos administrativos); la ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>2027-02-14</t>
         </is>
       </c>
-      <c r="M41" s="2" t="inlineStr">
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>categoría de algunos hoteles; número de algunos vuelos; itinerario día por día (la ficha no lo tiene)</t>
         </is>
       </c>
-      <c r="N41" s="2" t="inlineStr"/>
       <c r="O41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3397,56 +3603,61 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
+          <t>AS-561135</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
           <t>https://allseasons.tourvector.com/espanol/paquete2/561135/Descubri-Buzios-con-JetSMART/194626755/</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>9 de enero 2027</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Búzios: Lestada Pousada · 7 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>JetSMART JA 3816 Buenos Aires (EZE) – Río de Janeiro 09/01/2027 12:54 – 15:50
 JetSMART JA 3817 Río de Janeiro – Buenos Aires (EZE) 16/01/2027 13:50 – 17:14</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>1 valija de 23 kg en bodega</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>Desde USD 1.500 (por persona en base doble — precio final con impuestos)
 Precio final por persona en base doble publicado por el operador: USD 1.500 (total 2 adultos USD 3.000). La ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>2027-01-09</t>
         </is>
       </c>
-      <c r="M42" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>categoría de hotel; confirmar que es precio de venta al público</t>
         </is>
       </c>
-      <c r="N42" s="2" t="inlineStr"/>
       <c r="O42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3466,56 +3677,61 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
+          <t>AS-561130</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
           <t>https://allseasons.tourvector.com/espanol/paquete2/561130/Disfruta-Rio-De-Janeiro-con-JetSMART/193847595/</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>9 de enero 2027</t>
         </is>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="G43" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Río de Janeiro (Copacabana): Windsor Martinique 3* · 7 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>JetSMART JA 3816 Buenos Aires (EZE) – Río de Janeiro 09/01/2027 12:54 – 15:50
 JetSMART JA 3817 Río de Janeiro – Buenos Aires (EZE) 16/01/2027 13:50 – 17:14</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="J43" s="2" t="inlineStr">
         <is>
           <t>1 valija de 23 kg en bodega</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>Desde USD 1.500 (por persona en base doble — precio final con impuestos)
 Precio final por persona en base doble publicado por el operador: USD 1.500 (total 2 adultos USD 3.000). La ficha no desglosa componentes.</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>2027-01-09</t>
         </is>
       </c>
-      <c r="M43" s="2" t="inlineStr">
+      <c r="N43" s="2" t="inlineStr">
         <is>
           <t>confirmar que es precio de venta al público</t>
         </is>
       </c>
-      <c r="N43" s="2" t="inlineStr"/>
       <c r="O43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3535,56 +3751,61 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
+          <t>AS-217217</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
           <t>https://allseasons.tourvector.com/espanol/paquete2/217217/Salvador-con-GOL/193685985/</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>9 de enero 2027</t>
         </is>
       </c>
-      <c r="F44" s="2" t="n">
+      <c r="G44" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Salvador de Bahía (Ondina): Vila Galé Salvador 5* · 7 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>GOL G3 7213 Buenos Aires (AEP) – Salvador (SSA) 09/01/2027 22:15 – 02:40 (+1)
 GOL G3 7212 Salvador (SSA) – Buenos Aires (AEP) 17/01/2027 03:10 – 08:00</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>1 valija de 23 kg en bodega</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>Desde USD 1.356 (por persona en base doble — precio final con impuestos)
 Precio final por persona en base doble publicado por el operador: USD 1.356 (total 2 adultos USD 2.712). La ficha no desglosa componentes. Otras salidas listadas sin precio: enero a marzo 2027.</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>2027-01-09</t>
         </is>
       </c>
-      <c r="M44" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>otras fechas sin precio; confirmar que es precio de venta al público</t>
         </is>
       </c>
-      <c r="N44" s="2" t="inlineStr"/>
       <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3604,56 +3825,61 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
+          <t>AS-322357</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
           <t>https://allseasons.tourvector.com/espanol/paquete2/322357/Arraial-DAjuda-con-GOL/194999179/</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>10 de enero 2027</t>
         </is>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="G45" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Arraial d'Ajuda: Pousada Coqueiros · 7 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>GOL G3 7493 Buenos Aires (EZE) – Porto Seguro (BPS) 10/01/2027 01:10 – 05:00
 GOL G3 7492 Porto Seguro (BPS) – Buenos Aires (EZE) 16/01/2027 23:00 – 03:10 (+1)</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>1 valija de 23 kg en bodega</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>Desde USD 1.739 (por persona en base doble — precio final con impuestos)
 Precio final por persona en base doble publicado por el operador: USD 1.739 (total 2 adultos USD 3.478). La ficha no desglosa componentes. Otras salidas listadas sin precio: 17/01/2027.</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>2027-01-10</t>
         </is>
       </c>
-      <c r="M45" s="2" t="inlineStr">
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>categoría de hotel; otras fechas sin precio; confirmar que es precio de venta al público</t>
         </is>
       </c>
-      <c r="N45" s="2" t="inlineStr"/>
       <c r="O45" s="2" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3673,56 +3899,61 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
+          <t>AS-118771</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
           <t>https://allseasons.tourvector.com/espanol/paquete2/118771/Descubri-Florianopolis-con-JetSMART/194950084/</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>16 de enero 2027</t>
         </is>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="G46" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Florianópolis (Ingleses): Porto Sol Ingleses · 7 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>JetSMART JA 3824 Buenos Aires (EZE) – Florianópolis (FLN) 16/01/2027 12:15 – 14:15
 JetSMART JA 3825 Florianópolis (FLN) – Buenos Aires (EZE) 23/01/2027 15:10 – 17:25</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>1 valija de 23 kg en bodega</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>Desde USD 1.480 (por persona en base doble — precio final con impuestos)
 Precio final por persona en base doble publicado por el operador: USD 1.480 (total 2 adultos USD 2.960). La ficha no desglosa componentes. Otras salidas listadas sin precio: 09/01/2027.</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="M46" s="2" t="inlineStr">
         <is>
           <t>2027-01-16</t>
         </is>
       </c>
-      <c r="M46" s="2" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>categoría de hotel; otras fechas sin precio; confirmar que es precio de venta al público</t>
         </is>
       </c>
-      <c r="N46" s="2" t="inlineStr"/>
       <c r="O46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3742,56 +3973,61 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
+          <t>AS-195199</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
           <t>https://allseasons.tourvector.com/espanol/paquete2/195199/Descubri-Maceio-con-LATAM/195126896/</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>26 de enero 2027</t>
         </is>
       </c>
-      <c r="F47" s="2" t="n">
+      <c r="G47" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Maceió: Ritz Suites Grand Hotel Boutique · 7 noches · Desayuno</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>LATAM LA 8163 Buenos Aires (EZE) – Maceió (MCZ) 26/01/2027 02:15 – 07:15
 LATAM LA 8162 Maceió (MCZ) – Buenos Aires (EZE) 02/02/2027 10:45 – 16:00</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>1 valija de 23 kg en bodega</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>Desde USD 1.511 (por persona en base doble — precio final con impuestos)
 Precio final por persona en base doble publicado por el operador: USD 1.511 (total 2 adultos USD 3.022). La ficha no desglosa componentes. Otras salidas listadas sin precio: 12/01/2027 y 19/01/2027.</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="M47" s="2" t="inlineStr">
         <is>
           <t>2027-01-26</t>
         </is>
       </c>
-      <c r="M47" s="2" t="inlineStr">
+      <c r="N47" s="2" t="inlineStr">
         <is>
           <t>categoría de hotel; otras fechas sin precio; confirmar que es precio de venta al público</t>
         </is>
       </c>
-      <c r="N47" s="2" t="inlineStr"/>
       <c r="O47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3809,57 +4045,62 @@
           <t>Praia do Forte — 20 de febrero 2027</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>AS-162781</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>20 de febrero 2027</t>
         </is>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="G48" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Praia do Forte: Iberostar Waves Bahia · 7 noches · All Inclusive</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>GOL G3 7213 Buenos Aires (AEP) – Salvador (SSA) 20/02/2027 22:00 – 02:10 (+1)
 GOL G3 7212 Salvador (SSA) – Buenos Aires (AEP) 28/02/2027 03:10 – 08:00</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>1 valija de 23 kg en bodega</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>Desde USD 2.537 (por persona en base doble — precio final con impuestos)
 Precio final por persona en base doble publicado por el operador: USD 2.537 (total 2 adultos USD 5.074). La ficha no desglosa componentes. Otras salidas listadas sin precio: enero a marzo 2027.</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>2027-02-20</t>
         </is>
       </c>
-      <c r="M48" s="2" t="inlineStr">
+      <c r="N48" s="2" t="inlineStr">
         <is>
           <t>categoría de hotel; otras fechas sin precio; confirmar que es precio de venta al público</t>
         </is>
       </c>
-      <c r="N48" s="2" t="inlineStr"/>
       <c r="O48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O48"/>
+  <autoFilter ref="A1:P48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
salvador-de-bahia-ene-2027 (AS-217217): precio corregido a USD 1.455 con Vila Galé Salvador (antes 1.356), a pedido del usuario
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -794,7 +794,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Vietnam, Camboya &amp; Tailandia 2027 — Salida grupal</t>
+          <t>Vietnam, Camboya y Tailandia — Salida grupal, 7 de marzo 2027</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hong Kong &amp; China 2027 — Salida grupal</t>
+          <t>Hong Kong y la China milenaria — Salida grupal, 10 de mayo 2027</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Malasia, Singapur &amp; Bali — Salida grupal</t>
+          <t>Malasia, Singapur y Bali — Salida grupal, 24 de mayo 2027</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Andalucía, Portugal, País Vasco y Lourdes — 6 de junio 2027</t>
+          <t>Andalucía, Portugal y País Vasco, con Lourdes — 6 de junio 2027</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Río de Janeiro — 9 de enero 2027</t>
+          <t>Río de Janeiro: verano en Copacabana — 9 de enero 2027</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -3785,8 +3785,8 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Desde USD 1.356 (por persona en base doble — precio final con impuestos)
-Precio final por persona en base doble publicado por el operador: USD 1.356 (total 2 adultos USD 2.712). La ficha no desglosa componentes. Otras salidas listadas sin precio: enero a marzo 2027.</t>
+          <t>Desde USD 1.455 (por persona en base doble — precio final con impuestos)
+Precio final por persona en base doble publicado por el operador: USD 1.455 (total 2 adultos USD 2.910). La ficha no desglosa componentes. Otras salidas listadas sin precio: enero a marzo 2027. Corregido el 19/10/2026 a pedido del usuario: el precio correcto con Vila Galé Salvador es USD 1.455 (antes figuraba 1.356).</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Praia do Forte — 20 de febrero 2027</t>
+          <t>Praia do Forte, all inclusive en Bahía — 20 de febrero 2027</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Parte 7b — Station (ST-5DC17AAC3394 Mendoza, ST-9ABEECA36365 Salta: findes largos 5 al 8/12/2026 con hotel a elección, ARS) y VieTur (VT-11825 Esencias del Perú 7/5/2027 USD 3.140, VT-11817 Búzios posada a elección 11/1/2027 USD 1.095); Bariloche: vigencia a 30 días (19/11/2026); fichas en data/fichas; fotos Pexels 31025236, 21336116, 16973651, 18988842; filas en la planilla de revisión; madre Latinoamérica con su primera salida
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4099,6 +4099,407 @@
       <c r="O48" s="2" t="inlineStr"/>
       <c r="P48" s="2" t="inlineStr"/>
     </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Bariloche, fin de semana largo · 5 al 8 de diciembre 2026</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>ST-F82F837EC63E</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://stationtravel.tur.ar/producto?id=F82F837EC63E</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>5 de diciembre 2026</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Bariloche: Hotel Nevada · 3 noches · Desayuno
+Bariloche: Huinid Pioneros Aparts · 3 noches · Desayuno
+Bariloche: Hotel Cristal Bariloche · 3 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>JetSMART JA 3043 Buenos Aires (EZE) – Bariloche (BRC) 05/12/2026 07:00 – 09:21
+JetSMART JA 3052 Bariloche (BRC) – Buenos Aires (EZE) 08/12/2026 23:26 – 01:34 (+1)</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>10 kg</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Desde ARS 699.030 (por persona en base doble · precio final)
+Precios por persona en base doble publicados por el operador como finales, según hotel del selector: Hotel Nevada ARS 699.030 (Desde), Huinid Pioneros Aparts ARS 867.080, Hotel Cristal Bariloche ARS 895.315. La ficha no desglosa componentes ni informa categoría de los hoteles. Leído con Playwright sin enviar formularios.</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hoteles</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="n"/>
+      <c r="P49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Mendoza, fin de semana largo con cupo aéreo · 5 al 8 de diciembre 2026</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>ST-5DC17AAC3394</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://stationtravel.tur.ar/producto?id=5DC17AAC3394</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>5 de diciembre 2026</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Mendoza: Hotel Carollo Gold · 3 noches · Desayuno
+Mendoza: Raíces Aconcagua · 3 noches · Desayuno
+Mendoza: Premium Tower Suites · 3 noches · Desayuno
+Mendoza: Amerian Executive Mendoza · 3 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>JetSMART JA 3626 Buenos Aires (AEP) – Mendoza (MDZ) 05/12/2026 14:00 – 15:55
+JetSMART JA 3075 Mendoza (MDZ) – Buenos Aires (AEP) 08/12/2026 22:40 – 00:21 (+1)</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>10 kg</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Desde ARS 541.899 (por persona en base doble · precio final)
+Precios por persona en base doble publicados por el operador como finales, según hotel del selector: Hotel Carollo Gold ARS 541.899 (Desde), Raíces Aconcagua ARS 629.810, Premium Tower Suites ARS 759.025, Amerian Executive Mendoza ARS 841.315. La ficha no desglosa componentes ni informa categoría de los hoteles. Leído con Playwright sin enviar formularios. Vigencia: 30 días desde la carga por ser nacional en ARS.</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hoteles</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="n"/>
+      <c r="P50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Salta, fin de semana largo con cupo aéreo · 5 al 8 de diciembre 2026</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>ST-9ABEECA36365</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://stationtravel.tur.ar/producto?id=9ABEECA36365</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>5 de diciembre 2026</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Salta: Hotel Marilian · 3 noches · Desayuno
+Salta: Hotel del Virrey · 3 noches · Desayuno
+Salta: Casa Real · 3 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Aerolíneas Argentinas AR 1488 Buenos Aires (AEP) – Salta (SLA) 05/12/2026 05:00 – 07:15
+Aerolíneas Argentinas AR 1501 Salta (SLA) – Buenos Aires (AEP) 08/12/2026 21:20 – 23:25</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>8 kg</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Desde ARS 710.845 (por persona en base doble · precio final)
+Página identificada como 'Cupo Confirmado Salta | Finde XXL | Salida 05 de Diciembre'. Precios por persona en base doble publicados por el operador como finales, según hotel del selector: Hotel Marilian ARS 710.845 (Desde), Hotel del Virrey ARS 839.560, Casa Real ARS 914.920. La ficha no desglosa componentes ni informa categoría de los hoteles. Leído con Playwright sin enviar formularios. Vigencia: 30 días desde la carga por ser nacional en ARS.</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hoteles</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="n"/>
+      <c r="P51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Latinoamérica</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Esencias del Perú, salida grupal acompañada · 7 de mayo 2027</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>VT-11825</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vietur.com.ar/circuitos/1/11825?product_type=2&amp;currency=USD</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>7 de mayo 2027</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Lima: Libre Hotel BW Signature Collection 3* · 2 noches · Desayuno
+Arequipa: Hotel Crismar by Xima Hotels 3* · 1 noches · Desayuno
+Colca: El Refugio Hotel · 1 noches · Desayuno
+Puno: Lake Titicaca · 2 noches · Desayuno
+Cusco: Terra Andina Mansion Colonial 4* · 3 noches · Desayuno
+Valle Sagrado: Augustos Valle · 1 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>LATAM LA 2976 Buenos Aires (EZE) – Lima (LIM) 07/05/2027 07:20 – 10:10
+LATAM LA 2103 Lima (LIM) – Arequipa (AQP) 09/05/2027 05:50 – 07:20
+LATAM LA 2293 Cusco (CUZ) – Lima (LIM) 17/05/2027 08:40 – 10:15
+LATAM LA 2369 Lima (LIM) – Buenos Aires (AEP) 17/05/2027 12:10 – 18:30</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Equipaje incluido</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 3.140 (por persona en base doble · total con impuestos)
+Panel de la salida 07/05/2027, categoría Turista: doble USD 2.430 + 710 tax = 3.140; single 2.915 + 760 = 3.675; triple 2.400 + 700 = 3.100; doble a compartir 2.670 + 740 = 3.410. Según legales, los TAX incluyen impuestos aéreos DNT, IVA terrestre, gastos administrativos y de reserva. Pagos en pesos: percepción 30% RG 5463 aparte (aéreo USD 173; terrestre DBL USD 415 / SGL 524 / DBL a compartir 470 / TPL 409). La web es para agencias y no marca el precio como neto ni comisionable: confirmar que es precio de venta al público. Noches por ciudad deducidas del itinerario (Lima 2, Arequipa 1, Colca 1, Puno 2, Cusco 3, Valle Sagrado 1). Leído con Playwright sin login ni formularios.
+single: USD 3.675
+triple: USD 3.100</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>categoría de 3 hoteles; peso del equipaje; confirmar precio de venta al público (web de agencias)</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="n"/>
+      <c r="P52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Búzios, posada a elección · 11 de enero 2027</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>VT-11817</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vietur.com.ar/circuitos/1/11817?product_type=8&amp;currency=USD</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>11 de enero 2027</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Búzios: Pousada Vila do Sol · 7 noches · Desayuno
+Búzios: Pousada Vila Pitanga · 7 noches · Desayuno
+Búzios: Gammel Dansk · 7 noches · Desayuno
+Búzios: Villa Mercedes · 7 noches · Desayuno
+Búzios: Pousada Villegaignon · 7 noches · Desayuno
+Búzios: Barra da Lagoa Hotel · 7 noches · Desayuno
+Búzios: Pousada Lestada · 7 noches · Desayuno
+Búzios: Pousada dos Tangarás · 7 noches · Desayuno
+Búzios: Bucaneiro · 7 noches · Desayuno
+Búzios: La Foret 3* · 7 noches · Desayuno
+Búzios: Armação dos Búzios Pousada Design · 7 noches · Desayuno
+Búzios: Ilha Branca Inn · 7 noches · Desayuno
+Búzios: Pousada La Chimere · 7 noches · Desayuno
+Búzios: La Boheme · 7 noches · Desayuno</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>LATAM LA 777 Buenos Aires (EZE) – Río de Janeiro (GIG) 11/01/2027 15:10 – 18:10
+LATAM LA 776 Río de Janeiro (GIG) – Buenos Aires (EZE) 18/01/2027 10:30 – 13:55</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Bolso de mano + carry on 12 kg</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 1.095 (por persona en base doble · total con impuestos)
+Panel de la salida 11/01/2027, precio por persona + USD 110 tax en todas las opciones. Base doble (tarifa / total): Pousada Vila do Sol 985 / 1095; Pousada Vila Pitanga 1105 / 1215; Gammel Dansk 1110 / 1220; Villa Mercedes 1110 / 1220; Pousada Villegaignon 1175 / 1285; Barra da Lagoa Hotel 1175 / 1285; Pousada Lestada 1195 / 1305; Pousada dos Tangarás 1230 / 1340; Bucaneiro 1240 / 1350; La Foret 1295 / 1405; Armação dos Búzios Pousada Design 1345 / 1455; Ilha Branca Inn 1385 / 1495; Pousada La Chimere 1505 / 1615; La Boheme 1695 / 1805. Single y triple de la posada Desde: 1.550 + 110 = 1.660 y 905 + 110 = 1.015. Los legales dicen que las tarifas no incluyen IVA ni gastos administrativos: se asume que el 'tax' de USD 110 los cubre; confirmar. Pagos en pesos: percepción 30% RG 5463 aparte (aéreo USD 85 y terrestre según posada). La web es para agencias y no marca el precio como neto ni comisionable: confirmar que es precio de venta al público. Existe buzios-ene-2027 (otro operador, 9/1/2027, USD 1.500): mismo destino y semana, distinto producto. Leído con Playwright sin login ni formularios.
+single: USD 1.660
+triple: USD 1.015</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-11</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>categoría de hoteles; confirmar que el tax USD 110 cubre IVA y gastos; confirmar precio de venta al público (web de agencias); ojo: ya existe buzios-ene-2027 (AS, 9/1/2027)</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="n"/>
+      <c r="P53" s="2" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ajuste parte 7: buzios-posadas-ene-2027 (VT-11817) pasa a activo=false hasta confirmar si el total incluye IVA y gastos administrativos (los legales no lo aclaran); esencias-del-peru-may-2027 sigue activo (la ficha dice que los TAX incluyen IVA terrestre, gastos administrativos y de reserva); planilla actualizada
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -4414,7 +4414,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>ACTIVO</t>
+          <t>INACTIVO</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>categoría de hoteles; confirmar que el tax USD 110 cubre IVA y gastos; confirmar precio de venta al público (web de agencias); ojo: ya existe buzios-ene-2027 (AS, 9/1/2027)</t>
+          <t>Falta confirmar si el total incluye IVA y gastos administrativos (los legales dicen que la tarifa no los incluye y no aclaran qué cubre el tax de USD 110); categoría de hoteles; confirmar precio de venta al público (web de agencias); ya existe buzios-ene-2027 (AS, 9/1/2027)</t>
         </is>
       </c>
       <c r="O53" s="2" t="n"/>

</xml_diff>

<commit_message>
Ajuste parte 7: buzios-posadas-ene-2027 (VT-11817) vuelve a activo con 5% estimado de IVA y gastos sobre tarifa + tax (Desde USD 1.150, single 1.743, triple 1.066; las 14 posadas con el mismo criterio); esencias-del-peru-may-2027 sin cambios (los TAX ya incluyen IVA y gastos según la ficha); planilla actualizada
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -4414,7 +4414,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>INACTIVO</t>
+          <t>ACTIVO</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -4476,10 +4476,9 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Desde USD 1.095 (por persona en base doble · total con impuestos)
-Panel de la salida 11/01/2027, precio por persona + USD 110 tax en todas las opciones. Base doble (tarifa / total): Pousada Vila do Sol 985 / 1095; Pousada Vila Pitanga 1105 / 1215; Gammel Dansk 1110 / 1220; Villa Mercedes 1110 / 1220; Pousada Villegaignon 1175 / 1285; Barra da Lagoa Hotel 1175 / 1285; Pousada Lestada 1195 / 1305; Pousada dos Tangarás 1230 / 1340; Bucaneiro 1240 / 1350; La Foret 1295 / 1405; Armação dos Búzios Pousada Design 1345 / 1455; Ilha Branca Inn 1385 / 1495; Pousada La Chimere 1505 / 1615; La Boheme 1695 / 1805. Single y triple de la posada Desde: 1.550 + 110 = 1.660 y 905 + 110 = 1.015. Los legales dicen que las tarifas no incluyen IVA ni gastos administrativos: se asume que el 'tax' de USD 110 los cubre; confirmar. Pagos en pesos: percepción 30% RG 5463 aparte (aéreo USD 85 y terrestre según posada). La web es para agencias y no marca el precio como neto ni comisionable: confirmar que es precio de venta al público. Existe buzios-ene-2027 (otro operador, 9/1/2027, USD 1.500): mismo destino y semana, distinto producto. Leído con Playwright sin login ni formularios.
-single: USD 1.660
-triple: USD 1.015</t>
+          <t>Desde USD 1.150 (por persona en base doble · total estimado con impuestos y gastos)
+Panel de la salida 11/01/2027: precio por persona + USD 110 tax en todas las opciones. Los legales dicen que las tarifas no incluyen IVA, gastos administrativos ni gastos de reserva y no dan el monto: por decisión del usuario (20/10/2026) se suma 5% sobre tarifa + tax, redondeando hacia arriba al dólar, como estimado a confirmar por el equipo. Desde (Pousada Vila do Sol): doble 985 + 110 + 5% = 1.150; single 1.550 + 110 + 5% = 1.743; triple 905 + 110 + 5% = 1.066. Base doble por posada (tarifa / total estimado): Pousada Vila do Sol 985 / 1150; Pousada Vila Pitanga 1105 / 1276; Gammel Dansk 1110 / 1281; Villa Mercedes 1110 / 1281; Pousada Villegaignon 1175 / 1350; Barra da Lagoa Hotel 1175 / 1350; Pousada Lestada 1195 / 1371; Pousada dos Tangarás 1230 / 1407; Bucaneiro 1240 / 1418; La Foret 1295 / 1476; Armação dos Búzios Pousada Design 1345 / 1528; Ilha Branca Inn 1385 / 1570; Pousada La Chimere 1505 / 1696; La Boheme 1695 / 1896. Pagos en pesos: percepción 30% RG 5463 aparte (aéreo USD 85 y terrestre según posada). La web es para agencias y no marca el precio como neto ni comisionable: confirmar que es precio de venta al público. Existe buzios-ene-2027 (otro operador, 9/1/2027, USD 1.500): mismo destino y semana, distinto producto. Leído con Playwright sin login ni formularios.
+single: USD 1.743 · triple: USD 1.066</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
@@ -4494,7 +4493,7 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>Falta confirmar si el total incluye IVA y gastos administrativos (los legales dicen que la tarifa no los incluye y no aclaran qué cubre el tax de USD 110); categoría de hoteles; confirmar precio de venta al público (web de agencias); ya existe buzios-ene-2027 (AS, 9/1/2027)</t>
+          <t>Confirmar total con IVA y gastos administrativos (5% estimado sobre tarifa + tax); categoría de hoteles; confirmar precio de venta al público (web de agencias); ya existe buzios-ene-2027 (AS, 9/1/2027)</t>
         </is>
       </c>
       <c r="O53" s="2" t="n"/>

</xml_diff>

<commit_message>
Parte 8 — cruceros de ida (DC-MAJ22 Majestic Princess Buenos Aires–Southampton 22 noches USD 1.808; DC-MAJ36 con fiordos noruegos 36 noches USD 4.531; DC-ZAA29 Zaandam Buenos Aires–Fort Lauderdale 29 noches USD 5.999): datos de capturas del buscador del operador, fichas en data/fichas, escalas como itinerario, aéreo de regreso no incluido, ETA UK / visa USA, vigencia 20/11/2026; fotos Pexels 5334261, 34203329, 38059196; filas en la planilla
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-paquetes-parte6.xlsx
+++ b/docs/revision-paquetes-parte6.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4499,6 +4499,222 @@
       <c r="O53" s="2" t="n"/>
       <c r="P53" s="2" t="n"/>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Cruceros</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Majestic Princess: de Buenos Aires a Southampton · 9 de febrero 2027</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>DC-MAJ22</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>capturas del buscador del operador</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>9 de febrero 2027 — embarque en Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Princess Cruises · Majestic Princess · escalas: Montevideo, Río de Janeiro, Las Palmas de Gran Canaria, Arrecife (Lanzarote), Santa Cruz de Tenerife, Casablanca, La Coruña</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>sin aéreo (crucero solo de ida; regreso a cotizar)</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 1.808 (por persona en base doble, cabina interior — impuestos incluidos)
+Interior: USD 1.808
+Balcón: USD 2.104
+Suite: USD 3.197
+Datos de capturas del buscador del operador transcriptos por el usuario el 21/10/2026 (el sitio del operador está bloqueado). Precios por pasajero con impuestos incluidos, cabina interior USD 1.808, balcón USD 2.104, suite USD 3.197 (exterior no disponible). Tarifas de promoción sin fecha: vigencia 30 días desde la carga. Faltantes: confirmar propinas, confirmar precio de venta al público, itinerario día por día. Termina en el Reino Unido: ETA obligatoria.</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>confirmar propinas; confirmar precio de venta al público; itinerario día por día</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="n"/>
+      <c r="P54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Cruceros</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Majestic Princess: Buenos Aires a Southampton con fiordos noruegos · 9 de febrero 2027</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>DC-MAJ36</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>capturas del buscador del operador</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>9 de febrero 2027 — embarque en Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Princess Cruises · Majestic Princess · escalas: Montevideo, Río de Janeiro, Las Palmas de Gran Canaria, Arrecife (Lanzarote), Santa Cruz de Tenerife, Casablanca, La Coruña, Alesund, Trondheim, Tromsø, Alta, Molde</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>sin aéreo (crucero solo de ida; regreso a cotizar)</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 4.531 (por persona en base doble, cabina interior — impuestos incluidos)
+Interior: USD 4.531
+Balcón: USD 5.107
+Suite: USD 7.237
+Datos de capturas del buscador del operador transcriptos por el usuario el 21/10/2026 (el sitio del operador está bloqueado). Precios por pasajero con impuestos incluidos, cabina interior USD 4.531, balcón USD 5.107, suite USD 7.237. Tarifas de promoción sin fecha: vigencia 30 días desde la carga. Faltantes: confirmar propinas, confirmar precio de venta al público, itinerario día por día. Termina en el Reino Unido: ETA obligatoria.</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>confirmar propinas; confirmar precio de venta al público; itinerario día por día</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="n"/>
+      <c r="P55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Cruceros</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Zaandam: de Buenos Aires a Fort Lauderdale · 13 de febrero 2027</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>DC-ZAA29</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>capturas del buscador del operador</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>13 de febrero 2027 — embarque en Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Holland America Line · Zaandam · escalas: Santos, Ilhabela, Río de Janeiro, Salvador, Recife, Fortaleza, Belém, Isla del Diablo, Bridgetown, Castries, Basseterre, San Juan</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>sin aéreo (crucero solo de ida; regreso a cotizar)</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Desde USD 5.999 (por persona en base doble, cabina interior — impuestos incluidos)
+Interior: USD 5.999
+Exterior: USD 7.099
+Suite: USD 12.899
+Datos de capturas del buscador del operador transcriptos por el usuario el 21/10/2026 (el sitio del operador está bloqueado). Precios por pasajero con impuestos incluidos, cabina interior USD 5.999, exterior USD 7.099, suite USD 12.899 (balcón no disponible). Tarifas de promoción sin fecha: vigencia 30 días desde la carga. Faltantes: confirmar propinas, confirmar precio de venta al público, itinerario día por día. Termina en Estados Unidos: visa obligatoria para pasaporte argentino.</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>confirmar propinas; confirmar precio de venta al público; itinerario día por día</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="n"/>
+      <c r="P56" s="2" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>